<commit_message>
[IMP] edi_import_match: first release
</commit_message>
<xml_diff>
--- a/edi_import_match/tests/data/test_update_phone.xlsx
+++ b/edi_import_match/tests/data/test_update_phone.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -31,6 +31,9 @@
   </si>
   <si>
     <t xml:space="preserve">phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">street2</t>
   </si>
   <si>
     <t xml:space="preserve">The Jackson Group</t>
@@ -119,11 +122,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -250,7 +253,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.17"/>
@@ -269,16 +272,19 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>